<commit_message>
Adjustmens of csv output
Adjusting all the modules for the final csv versions
</commit_message>
<xml_diff>
--- a/data/benchmark_studies.xlsx
+++ b/data/benchmark_studies.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Benchmarks" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -654,49 +654,6 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>2024</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>IP / Licensing</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Royalty Rate (% of Net Sales)</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="G6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H6" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I6" t="n">
-        <v>9</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Comparable Uncontrolled Royalty Database 2024</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
         <v>2024</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deep code review: remove dead code, fix role-pair bug, add integration tests
</commit_message>
<xml_diff>
--- a/data/benchmark_studies.xlsx
+++ b/data/benchmark_studies.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Benchmarks" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>